<commit_message>
v5.19: report, test_interface_d_e_shapes covers 7 _Prod names, check workbook Q1 per-GPU basis and GM205 text
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FNE52EBh4awAQ4XsaZpE4F
</commit_message>
<xml_diff>
--- a/docs/reports/20261006_v5.19_查核.xlsx
+++ b/docs/reports/20261006_v5.19_查核.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>開放權重可比對象：Llama 3.1 405B 126 層、DeepSeek V3 61 層（arxiv 2507.14397 LIMINAL 等轉載；另一來源列 Llama 3.1 405B 為 80 層，兩源衝突）</t>
+          <t>開放權重可比對象：Llama 3.1 405B 126 層、DeepSeek V3 61 層（arxiv 2507.14397 LIMINAL 等轉載）</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>找到（整體吞吐，非 η_d 直接值）</t>
+          <t>找到（每 GPU 口徑可比；非 η_d 直接值）</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -993,12 +993,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>MLPerf Inference v6.1（2026-09-16，preview）DeepSeek-R1：VR NVL72 最高 2.5× GB300 NVL72（NVIDIA，Interested-party）；每 GPU 換算 1.6–2×；Qwen3-VL 最高 3.7×；NVFP4；ISL／OSL、互動性未讀到。InferenceX AgentX：160 tok/s/user 下每 MW 最高 30× GB300（NVIDIA 技術部落格 2026-08-24 摘要）</t>
+          <t>MLPerf Inference v6.1（2026-09-16，preview 類）DeepSeek-R1：VR NVL72 最高 2.5× GB300 NVL72（NVIDIA 宣稱，Interested-party）；依公布數字換算每 GPU 約 1.6–2×（Nebius 換算；本輪只讀到 remio.ai 摘要轉述，未讀 Nebius 原文）；NVFP4；ISL／OSL、互動性未讀到。另：Qwen3-VL 最高 3.7×；InferenceX AgentX 160 tok/s/user 下每 MW 最高 30×（NVIDIA 技術部落格摘要，口徑不同，不比）</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>本模型 VR200÷GB300 每 GW 產出（Sol）＝1.565×（Checks 第 20 列）、第 24 列對 MLPerf 比 2.53／2.57。MLPerf 每 GPU 1.6–2.5× 在或高於模型值 → 方向上支持 η_d 倍數 ≥1.0；不構成可直接代入的 η_d（吞吐比含峰值提升）</t>
+          <t>每 GPU 口徑比較：模型 VR200÷GB300（對 MLPerf，Checks 第 24 列）＝2.525×；NVIDIA 宣稱 2.5×（廠商，偏樂觀端）；第三方每 GPU 換算 1.6–2×。模型與廠商宣稱一致，但高於第三方換算 26–58%（2.525/2.0＝1.26；2.525/1.6＝1.58）。結論：方向上支持 F67 低端，模型可能高估 VR200（非單點結論：preview 類、廠商提交、換算口徑未讀原文）。（前版以每 GW 產出 1.565× 比對，口徑不同，已撤回）</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>preview 類、廠商提交（Interested-party）；需第二來源</t>
+          <t>未找到 prefill／η_d 的直接值；需第二來源（非廠商）與原文</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.19: Q1 rewritten on same-basis interactive comparison (model 2.525x vs MLPerf v6.1 2.575x); report text aligned
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FNE52EBh4awAQ4XsaZpE4F
</commit_message>
<xml_diff>
--- a/docs/reports/20261006_v5.19_查核.xlsx
+++ b/docs/reports/20261006_v5.19_查核.xlsx
@@ -915,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>找到（每 GPU 口徑可比；非 η_d 直接值）</t>
+          <t>找到（同口徑 interactive 已在模型內；非 η_d 直接值）</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -993,12 +993,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>MLPerf Inference v6.1（2026-09-16，preview 類）DeepSeek-R1：VR NVL72 最高 2.5× GB300 NVL72（NVIDIA 宣稱，Interested-party）；依公布數字換算每 GPU 約 1.6–2×（Nebius 換算；本輪只讀到 remio.ai 摘要轉述，未讀 Nebius 原文）；NVFP4；ISL／OSL、互動性未讀到。另：Qwen3-VL 最高 3.7×；InferenceX AgentX 160 tok/s/user 下每 MW 最高 30×（NVIDIA 技術部落格摘要，口徑不同，不比）</t>
+          <t>同口徑：MLPerf Inference v6.1（2026-09-16，preview 類）DeepSeek-R1 interactive，VR200÷GB300＝2.575×（Calib 第 151 列；NVIDIA 宣稱最高 2.5×，Interested-party）。待查證據：Nebius 依公布數字換算每 GPU 約 1.6–2×——情境與規模不同，原文未讀（本輪只見 remio.ai 摘要轉述）。NVFP4；ISL／OSL 未讀到</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>每 GPU 口徑比較：模型 VR200÷GB300（對 MLPerf，Checks 第 24 列）＝2.525×；NVIDIA 宣稱 2.5×（廠商，偏樂觀端）；第三方每 GPU 換算 1.6–2×。模型與廠商宣稱一致，但高於第三方換算 26–58%（2.525/2.0＝1.26；2.525/1.6＝1.58）。結論：方向上支持 F67 低端，模型可能高估 VR200（非單點結論：preview 類、廠商提交、換算口徑未讀原文）。（前版以每 GW 產出 1.565× 比對，口徑不同，已撤回）</t>
+          <t>同口徑 interactive：模型 VR200÷GB300＝2.525×（Calib 第 150 列、Checks 第 24 列）對 MLPerf v6.1 2.575×（第 151 列），差 −1.9%，支持 F67≈1.0（沿用 GB300 效率係數）。Nebius 每 GPU 1.6–2× 若屬實，則指向 F67 低端（模型可能高估 VR200），但情境與規模不同、原文未讀，只列為低端的待查證據，不作結論。</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1008,7 +1008,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>未找到 prefill／η_d 的直接值；需第二來源（非廠商）與原文</t>
+          <t>搜尋摘要，原文未讀（Nebius 換算未讀原文）</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>需讀 MLPerf v6.1 原始提交與 Nebius 原文，確認情境（interactive／server／offline）與 GPU 數</t>
         </is>
       </c>
     </row>

</xml_diff>